<commit_message>
feat: implement practice plan printing, local downloading, and improved database plan parsing logic
</commit_message>
<xml_diff>
--- a/BHS_Schedule.xlsx
+++ b/BHS_Schedule.xlsx
@@ -1,44 +1,141 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr codeName="ThisWorkbook"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Source\repos\BHS-Soccer\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82FB674C-FFD3-42F1-9D7C-97E9F7C6A250}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
     <sheet name="Schedule" sheetId="1" r:id="rId1"/>
   </sheets>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
-<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
-  <metadataTypes count="1">
-    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
-  </metadataTypes>
-  <futureMetadata name="XLDAPR" count="1">
-    <bk>
-      <extLst>
-        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
-          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
-        </ext>
-      </extLst>
-    </bk>
-  </futureMetadata>
-  <cellMetadata count="1">
-    <bk>
-      <rc t="1" v="0"/>
-    </bk>
-  </cellMetadata>
-</metadata>
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="28">
+  <si>
+    <t>Date</t>
+  </si>
+  <si>
+    <t>Time</t>
+  </si>
+  <si>
+    <t>Opponent</t>
+  </si>
+  <si>
+    <t>Location</t>
+  </si>
+  <si>
+    <t>Home</t>
+  </si>
+  <si>
+    <t>Status</t>
+  </si>
+  <si>
+    <t>Score</t>
+  </si>
+  <si>
+    <t>AUG 12, 2026</t>
+  </si>
+  <si>
+    <t>6:30 PM</t>
+  </si>
+  <si>
+    <t>Yucaipa Thunderbirds</t>
+  </si>
+  <si>
+    <t>Home - Cougar Stadium</t>
+  </si>
+  <si>
+    <t>UPCOMING</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>AUG 18, 2026</t>
+  </si>
+  <si>
+    <t>5:00 PM</t>
+  </si>
+  <si>
+    <t>Citrus Valley Blackhawks</t>
+  </si>
+  <si>
+    <t>Away - Redlands, CA</t>
+  </si>
+  <si>
+    <t>Away</t>
+  </si>
+  <si>
+    <t>JUL 28, 2026</t>
+  </si>
+  <si>
+    <t>FINAL</t>
+  </si>
+  <si>
+    <t>Redlands East Valley</t>
+  </si>
+  <si>
+    <t>COMPLETED</t>
+  </si>
+  <si>
+    <t>3 - 1</t>
+  </si>
+  <si>
+    <t>JUL 22, 2026</t>
+  </si>
+  <si>
+    <t>Palm Springs Indians</t>
+  </si>
+  <si>
+    <t>Away - Palm Springs</t>
+  </si>
+  <si>
+    <t>2 - 0</t>
+  </si>
+  <si>
+    <t>2-0</t>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
+    <numFmt numFmtId="167" formatCode="[$-409]mmmm\ d\,\ yyyy;@"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -64,14 +161,26 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+  <cellXfs count="5">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -396,127 +505,201 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G5"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:G8"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="13.83203125" style="3" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="21.1640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="20.33203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="5.25" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>Date</v>
-      </c>
-      <c r="B1" t="str">
-        <v>Time</v>
-      </c>
-      <c r="C1" t="str">
-        <v>Opponent</v>
-      </c>
-      <c r="D1" t="str">
-        <v>Location</v>
-      </c>
-      <c r="E1" t="str">
-        <v>Home</v>
-      </c>
-      <c r="F1" t="str">
-        <v>Status</v>
-      </c>
-      <c r="G1" t="str">
-        <v>Score</v>
+    <row r="1" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A1" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" t="s">
+        <v>6</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>AUG 12, 2026</v>
-      </c>
-      <c r="B2" t="str">
-        <v>6:30 PM</v>
-      </c>
-      <c r="C2" t="str">
-        <v>Yucaipa Thunderbirds</v>
-      </c>
-      <c r="D2" t="str">
-        <v>Home - Cougar Stadium</v>
-      </c>
-      <c r="E2" t="str">
-        <v>Home</v>
-      </c>
-      <c r="F2" t="str">
-        <v>UPCOMING</v>
-      </c>
-      <c r="G2" t="str">
-        <v/>
+    <row r="2" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A2" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E2" t="s">
+        <v>4</v>
+      </c>
+      <c r="F2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G2" t="s">
+        <v>12</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>AUG 18, 2026</v>
-      </c>
-      <c r="B3" t="str">
-        <v>5:00 PM</v>
-      </c>
-      <c r="C3" t="str">
-        <v>Citrus Valley Blackhawks</v>
-      </c>
-      <c r="D3" t="str">
-        <v>Away - Redlands, CA</v>
-      </c>
-      <c r="E3" t="str">
-        <v>Away</v>
-      </c>
-      <c r="F3" t="str">
-        <v>UPCOMING</v>
-      </c>
-      <c r="G3" t="str">
-        <v/>
+    <row r="3" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A3" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="B3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D3" t="s">
+        <v>16</v>
+      </c>
+      <c r="E3" t="s">
+        <v>17</v>
+      </c>
+      <c r="F3" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3" t="s">
+        <v>12</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>JUL 28, 2026</v>
-      </c>
-      <c r="B4" t="str">
-        <v>FINAL</v>
-      </c>
-      <c r="C4" t="str">
-        <v>Redlands East Valley</v>
-      </c>
-      <c r="D4" t="str">
-        <v>Home - Cougar Stadium</v>
-      </c>
-      <c r="E4" t="str">
-        <v>Home</v>
-      </c>
-      <c r="F4" t="str">
-        <v>COMPLETED</v>
-      </c>
-      <c r="G4" t="str">
-        <v>3 - 1</v>
+    <row r="4" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A4" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="B4" t="s">
+        <v>19</v>
+      </c>
+      <c r="C4" t="s">
+        <v>20</v>
+      </c>
+      <c r="D4" t="s">
+        <v>10</v>
+      </c>
+      <c r="E4" t="s">
+        <v>4</v>
+      </c>
+      <c r="F4" t="s">
+        <v>21</v>
+      </c>
+      <c r="G4" t="s">
+        <v>22</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>JUL 22, 2026</v>
-      </c>
-      <c r="B5" t="str">
-        <v>FINAL</v>
-      </c>
-      <c r="C5" t="str">
-        <v>Palm Springs Indians</v>
-      </c>
-      <c r="D5" t="str">
-        <v>Away - Palm Springs</v>
-      </c>
-      <c r="E5" t="str">
-        <v>Away</v>
-      </c>
-      <c r="F5" t="str">
-        <v>COMPLETED</v>
-      </c>
-      <c r="G5" t="str">
-        <v>2 - 0</v>
+    <row r="5" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A5" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="B5" t="s">
+        <v>19</v>
+      </c>
+      <c r="C5" t="s">
+        <v>24</v>
+      </c>
+      <c r="D5" t="s">
+        <v>25</v>
+      </c>
+      <c r="E5" t="s">
+        <v>17</v>
+      </c>
+      <c r="F5" t="s">
+        <v>21</v>
+      </c>
+      <c r="G5" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A6" s="4">
+        <v>46230</v>
+      </c>
+      <c r="B6" t="s">
+        <v>14</v>
+      </c>
+      <c r="C6" t="s">
+        <v>15</v>
+      </c>
+      <c r="D6" t="s">
+        <v>10</v>
+      </c>
+      <c r="E6" t="s">
+        <v>4</v>
+      </c>
+      <c r="F6" t="s">
+        <v>21</v>
+      </c>
+      <c r="G6" s="1">
+        <v>46057</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A7" s="4">
+        <v>46621</v>
+      </c>
+      <c r="B7" t="s">
+        <v>14</v>
+      </c>
+      <c r="C7" t="s">
+        <v>20</v>
+      </c>
+      <c r="D7" t="s">
+        <v>17</v>
+      </c>
+      <c r="E7" t="s">
+        <v>17</v>
+      </c>
+      <c r="F7" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A8" s="4">
+        <v>46262</v>
+      </c>
+      <c r="B8" t="s">
+        <v>14</v>
+      </c>
+      <c r="C8" t="s">
+        <v>9</v>
+      </c>
+      <c r="D8" t="s">
+        <v>10</v>
+      </c>
+      <c r="E8" t="s">
+        <v>4</v>
+      </c>
+      <c r="F8" t="s">
+        <v>21</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>27</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G5"/>
+    <ignoredError sqref="A1:G2 A4:G5 A3:B3 D3:G3" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>